<commit_message>
Actualizados excel y memoria para subir
</commit_message>
<xml_diff>
--- a/IS2-Proyecto-Equipo-9-Trabajo.xlsx
+++ b/IS2-Proyecto-Equipo-9-Trabajo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="62">
   <si>
     <t>Factor de calificación</t>
   </si>
@@ -37,9 +37,6 @@
   </si>
   <si>
     <t>David Ferreras</t>
-  </si>
-  <si>
-    <t>Natalia Casarín</t>
   </si>
   <si>
     <t>Clases</t>
@@ -90,10 +87,16 @@
     <t>D/C-80</t>
   </si>
   <si>
+    <t>Otros métodos, si existen</t>
+  </si>
+  <si>
+    <t>D/C</t>
+  </si>
+  <si>
     <t>Factura</t>
   </si>
   <si>
-    <t>D/C</t>
+    <t>D-50/C-50</t>
   </si>
   <si>
     <t>LeerTodos</t>
@@ -102,10 +105,7 @@
     <t>Leer1</t>
   </si>
   <si>
-    <t>Otros métodos, si existen</t>
-  </si>
-  <si>
-    <t>C</t>
+    <t>C-50</t>
   </si>
   <si>
     <t>Dependiente</t>
@@ -144,6 +144,27 @@
     <t>Otros métodos</t>
   </si>
   <si>
+    <t>Venta</t>
+  </si>
+  <si>
+    <t>Abrir</t>
+  </si>
+  <si>
+    <t>D/C-10</t>
+  </si>
+  <si>
+    <t>Cerrar</t>
+  </si>
+  <si>
+    <t>LeerTodas</t>
+  </si>
+  <si>
+    <t>LeerUna</t>
+  </si>
+  <si>
+    <t>AñadirProducto</t>
+  </si>
+  <si>
     <t>Indicar los patrones GoF usados</t>
   </si>
   <si>
@@ -153,13 +174,16 @@
     <t>Singleton</t>
   </si>
   <si>
-    <t>Aplicado en las clases</t>
+    <t>Aplicado de forma general en las clases</t>
   </si>
   <si>
-    <t>BDConexion</t>
+    <t>BDConexion y controladores</t>
   </si>
   <si>
     <t>MVC</t>
+  </si>
+  <si>
+    <t>Aplicado de forma generalen las clases</t>
   </si>
   <si>
     <t>Controladores y vistas</t>
@@ -169,6 +193,15 @@
   </si>
   <si>
     <t>Integracion</t>
+  </si>
+  <si>
+    <t>Method Template</t>
+  </si>
+  <si>
+    <t>Aplicado en la clase TProducto y sus subclases</t>
+  </si>
+  <si>
+    <t>Negocio</t>
   </si>
 </sst>
 </file>
@@ -258,7 +291,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -319,6 +352,13 @@
     <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -534,7 +574,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="15.9"/>
     <col customWidth="1" min="2" max="2" width="12.4"/>
-    <col customWidth="1" min="3" max="3" width="28.1"/>
+    <col customWidth="1" min="3" max="3" width="40.2"/>
     <col customWidth="1" min="4" max="4" width="17.7"/>
     <col customWidth="1" min="5" max="5" width="16.5"/>
     <col customWidth="1" min="6" max="6" width="10.8"/>
@@ -590,9 +630,7 @@
       <c r="G2" s="3">
         <v>1.25</v>
       </c>
-      <c r="H2" s="3">
-        <v>1.0</v>
-      </c>
+      <c r="H2" s="3"/>
       <c r="I2" s="4"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
@@ -632,9 +670,7 @@
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>7</v>
-      </c>
+      <c r="H3" s="6"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
@@ -656,7 +692,7 @@
     </row>
     <row r="4" ht="18.0" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -715,26 +751,24 @@
     <row r="6" ht="18.0" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="D6" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>11</v>
+      <c r="G6" s="9" t="s">
+        <v>10</v>
       </c>
-      <c r="F6" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>11</v>
-      </c>
+      <c r="H6" s="9"/>
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1"/>
@@ -746,13 +780,13 @@
       <c r="A7" s="1"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>14</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>15</v>
       </c>
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
@@ -765,13 +799,13 @@
       <c r="A8" s="1"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
@@ -783,19 +817,19 @@
     <row r="9" ht="18.0" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="E9" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>20</v>
-      </c>
       <c r="G9" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
@@ -808,13 +842,13 @@
       <c r="A10" s="1"/>
       <c r="B10" s="10"/>
       <c r="C10" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="F10" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>23</v>
       </c>
       <c r="G10" s="9"/>
       <c r="U10" s="1"/>
@@ -827,7 +861,12 @@
     <row r="11" ht="18.0" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
+      <c r="C11" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>24</v>
+      </c>
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
@@ -888,26 +927,24 @@
     <row r="15" ht="18.0" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
-      <c r="H15" s="16" t="s">
-        <v>11</v>
-      </c>
+      <c r="H15" s="16"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
@@ -931,11 +968,13 @@
       <c r="A16" s="1"/>
       <c r="B16" s="17"/>
       <c r="C16" s="17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
-      <c r="D16" s="1"/>
+      <c r="D16" s="16" t="s">
+        <v>26</v>
+      </c>
       <c r="E16" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
@@ -963,11 +1002,13 @@
       <c r="A17" s="1"/>
       <c r="B17" s="17"/>
       <c r="C17" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
-      <c r="D17" s="1"/>
+      <c r="D17" s="16" t="s">
+        <v>26</v>
+      </c>
       <c r="E17" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -994,14 +1035,16 @@
     <row r="18" ht="18.0" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="17" t="s">
-        <v>18</v>
+      <c r="D18" s="16" t="s">
+        <v>26</v>
       </c>
-      <c r="D18" s="1"/>
       <c r="E18" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
@@ -1029,11 +1072,13 @@
       <c r="A19" s="1"/>
       <c r="B19" s="17"/>
       <c r="C19" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="1"/>
       <c r="E19" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
@@ -1061,11 +1106,13 @@
       <c r="A20" s="1"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
-      <c r="D20" s="1"/>
+      <c r="D20" s="16" t="s">
+        <v>26</v>
+      </c>
       <c r="E20" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -1093,9 +1140,11 @@
       <c r="A21" s="1"/>
       <c r="B21" s="17"/>
       <c r="C21" s="17" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
-      <c r="D21" s="1"/>
+      <c r="D21" s="16" t="s">
+        <v>29</v>
+      </c>
       <c r="E21" s="16" t="s">
         <v>29</v>
       </c>
@@ -1183,21 +1232,19 @@
         <v>30</v>
       </c>
       <c r="C24" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" s="16" t="s">
-        <v>11</v>
-      </c>
       <c r="F24" s="16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G24" s="1"/>
-      <c r="H24" s="16" t="s">
-        <v>11</v>
-      </c>
+      <c r="H24" s="16"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
@@ -1221,7 +1268,7 @@
       <c r="A25" s="1"/>
       <c r="B25" s="17"/>
       <c r="C25" s="17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D25" s="16" t="s">
         <v>31</v>
@@ -1229,7 +1276,7 @@
       <c r="E25" s="13"/>
       <c r="F25" s="1"/>
       <c r="G25" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -1255,7 +1302,7 @@
       <c r="A26" s="1"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D26" s="16" t="s">
         <v>32</v>
@@ -1288,13 +1335,13 @@
     <row r="27" ht="18.0" customHeight="1">
       <c r="A27" s="1"/>
       <c r="B27" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="17" t="s">
-        <v>18</v>
-      </c>
       <c r="D27" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E27" s="16"/>
       <c r="F27" s="1"/>
@@ -1323,10 +1370,10 @@
       <c r="A28" s="1"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E28" s="13"/>
       <c r="F28" s="1"/>
@@ -1389,11 +1436,11 @@
       <c r="A30" s="1"/>
       <c r="B30" s="17"/>
       <c r="C30" s="17" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
@@ -1479,23 +1526,21 @@
         <v>37</v>
       </c>
       <c r="C33" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D33" s="16" t="s">
+      <c r="E33" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="G33" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="E33" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F33" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="G33" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H33" s="16" t="s">
-        <v>11</v>
-      </c>
+      <c r="H33" s="16"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
@@ -1519,13 +1564,13 @@
       <c r="A34" s="1"/>
       <c r="B34" s="17"/>
       <c r="C34" s="19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="20"/>
       <c r="F34" s="16"/>
       <c r="G34" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
@@ -1551,13 +1596,13 @@
       <c r="A35" s="1"/>
       <c r="B35" s="17"/>
       <c r="C35" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="13"/>
       <c r="F35" s="1"/>
       <c r="G35" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
@@ -1582,16 +1627,16 @@
     <row r="36" ht="18.0" customHeight="1">
       <c r="A36" s="1"/>
       <c r="B36" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="13"/>
       <c r="F36" s="1"/>
       <c r="G36" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
@@ -1617,13 +1662,13 @@
       <c r="A37" s="1"/>
       <c r="B37" s="17"/>
       <c r="C37" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="13"/>
       <c r="F37" s="1"/>
       <c r="G37" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
@@ -1649,13 +1694,13 @@
       <c r="A38" s="1"/>
       <c r="B38" s="17"/>
       <c r="C38" s="19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="13"/>
       <c r="F38" s="1"/>
       <c r="G38" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
@@ -1681,7 +1726,7 @@
       <c r="A39" s="1"/>
       <c r="B39" s="17"/>
       <c r="C39" s="19" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D39" s="1"/>
       <c r="E39" s="16" t="s">
@@ -1768,23 +1813,21 @@
         <v>40</v>
       </c>
       <c r="C42" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D42" s="9" t="s">
-        <v>11</v>
-      </c>
       <c r="E42" s="16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
-      <c r="H42" s="9" t="s">
-        <v>12</v>
-      </c>
+      <c r="H42" s="9"/>
       <c r="I42" s="1"/>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
@@ -1807,18 +1850,16 @@
     <row r="43" ht="18.0" customHeight="1">
       <c r="A43" s="1"/>
       <c r="B43" s="21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
-      <c r="H43" s="16" t="s">
-        <v>25</v>
-      </c>
+      <c r="H43" s="16"/>
       <c r="I43" s="1"/>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
@@ -1842,15 +1883,13 @@
       <c r="A44" s="1"/>
       <c r="B44" s="10"/>
       <c r="C44" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
-      <c r="H44" s="16" t="s">
-        <v>25</v>
-      </c>
+      <c r="H44" s="16"/>
       <c r="I44" s="1"/>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
@@ -1874,15 +1913,13 @@
       <c r="A45" s="1"/>
       <c r="B45" s="10"/>
       <c r="C45" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
-      <c r="H45" s="16" t="s">
-        <v>25</v>
-      </c>
+      <c r="H45" s="16"/>
       <c r="I45" s="1"/>
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
@@ -1912,9 +1949,7 @@
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
-      <c r="H46" s="16" t="s">
-        <v>25</v>
-      </c>
+      <c r="H46" s="16"/>
       <c r="I46" s="1"/>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
@@ -1960,8 +1995,6 @@
       <c r="Z47" s="1"/>
     </row>
     <row r="48" ht="18.0" customHeight="1">
-      <c r="A48" s="1"/>
-      <c r="D48" s="1"/>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
@@ -1986,16 +2019,26 @@
       <c r="Z48" s="1"/>
     </row>
     <row r="49" ht="18.0" customHeight="1">
-      <c r="A49" s="13" t="s">
+      <c r="A49" s="22"/>
+      <c r="B49" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1"/>
-      <c r="G49" s="1"/>
-      <c r="H49" s="1"/>
+      <c r="C49" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F49" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="G49" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="H49" s="16"/>
       <c r="I49" s="1"/>
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
@@ -2016,19 +2059,19 @@
       <c r="Z49" s="1"/>
     </row>
     <row r="50" ht="18.0" customHeight="1">
-      <c r="A50" s="7" t="s">
+      <c r="A50" s="24"/>
+      <c r="B50" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C50" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B50" s="16" t="s">
+      <c r="D50" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="E50" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C50" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D50" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="E50" s="1"/>
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
@@ -2052,17 +2095,17 @@
       <c r="Z50" s="1"/>
     </row>
     <row r="51" ht="18.0" customHeight="1">
-      <c r="A51" s="1"/>
-      <c r="B51" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="C51" s="1" t="s">
+      <c r="A51" s="24"/>
+      <c r="B51" s="26"/>
+      <c r="C51" s="19" t="s">
         <v>45</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
-      <c r="E51" s="1"/>
+      <c r="E51" s="16" t="s">
+        <v>44</v>
+      </c>
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
@@ -2086,16 +2129,17 @@
       <c r="Z51" s="1"/>
     </row>
     <row r="52" ht="18.0" customHeight="1">
-      <c r="B52" s="9" t="s">
-        <v>49</v>
+      <c r="A52" s="24"/>
+      <c r="B52" s="26"/>
+      <c r="C52" s="19" t="s">
+        <v>46</v>
       </c>
-      <c r="C52" s="9" t="s">
-        <v>45</v>
+      <c r="D52" s="16" t="s">
+        <v>35</v>
       </c>
-      <c r="D52" s="9" t="s">
-        <v>50</v>
+      <c r="E52" s="16" t="s">
+        <v>44</v>
       </c>
-      <c r="E52" s="1"/>
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
@@ -2119,7 +2163,17 @@
       <c r="Z52" s="1"/>
     </row>
     <row r="53" ht="18.0" customHeight="1">
-      <c r="E53" s="1"/>
+      <c r="A53" s="24"/>
+      <c r="B53" s="26"/>
+      <c r="C53" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D53" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="E53" s="16" t="s">
+        <v>44</v>
+      </c>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
@@ -2143,11 +2197,17 @@
       <c r="Z53" s="1"/>
     </row>
     <row r="54" ht="18.0" customHeight="1">
-      <c r="A54" s="1"/>
-      <c r="B54" s="1"/>
-      <c r="C54" s="1"/>
-      <c r="D54" s="1"/>
-      <c r="E54" s="1"/>
+      <c r="A54" s="24"/>
+      <c r="B54" s="26"/>
+      <c r="C54" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="D54" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="E54" s="16" t="s">
+        <v>44</v>
+      </c>
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
@@ -2171,11 +2231,16 @@
       <c r="Z54" s="1"/>
     </row>
     <row r="55" ht="18.0" customHeight="1">
-      <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="1"/>
-      <c r="E55" s="1"/>
+      <c r="B55" s="17"/>
+      <c r="C55" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D55" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="E55" s="16" t="s">
+        <v>44</v>
+      </c>
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
@@ -2199,10 +2264,7 @@
       <c r="Z55" s="1"/>
     </row>
     <row r="56" ht="18.0" customHeight="1">
-      <c r="A56" s="1"/>
-      <c r="B56" s="1"/>
-      <c r="C56" s="1"/>
-      <c r="D56" s="1"/>
+      <c r="D56" s="16"/>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
@@ -2227,10 +2289,6 @@
       <c r="Z56" s="1"/>
     </row>
     <row r="57" ht="18.0" customHeight="1">
-      <c r="A57" s="1"/>
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="1"/>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
@@ -2255,7 +2313,9 @@
       <c r="Z57" s="1"/>
     </row>
     <row r="58" ht="18.0" customHeight="1">
-      <c r="A58" s="1"/>
+      <c r="A58" s="13" t="s">
+        <v>49</v>
+      </c>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
@@ -2283,10 +2343,18 @@
       <c r="Z58" s="1"/>
     </row>
     <row r="59" ht="18.0" customHeight="1">
-      <c r="A59" s="1"/>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-      <c r="D59" s="1"/>
+      <c r="A59" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B59" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C59" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D59" s="16" t="s">
+        <v>53</v>
+      </c>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
       <c r="G59" s="1"/>
@@ -2312,9 +2380,15 @@
     </row>
     <row r="60" ht="18.0" customHeight="1">
       <c r="A60" s="1"/>
-      <c r="B60" s="1"/>
-      <c r="C60" s="1"/>
-      <c r="D60" s="1"/>
+      <c r="B60" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C60" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D60" s="16" t="s">
+        <v>56</v>
+      </c>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
@@ -2339,10 +2413,15 @@
       <c r="Z60" s="1"/>
     </row>
     <row r="61" ht="18.0" customHeight="1">
-      <c r="A61" s="1"/>
-      <c r="B61" s="1"/>
-      <c r="C61" s="1"/>
-      <c r="D61" s="1"/>
+      <c r="B61" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>58</v>
+      </c>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
@@ -2368,9 +2447,15 @@
     </row>
     <row r="62" ht="18.0" customHeight="1">
       <c r="A62" s="1"/>
-      <c r="B62" s="1"/>
-      <c r="C62" s="1"/>
-      <c r="D62" s="1"/>
+      <c r="B62" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C62" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="D62" s="16" t="s">
+        <v>61</v>
+      </c>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>

</xml_diff>